<commit_message>
Add Claude Opus 4.5 Judgements
</commit_message>
<xml_diff>
--- a/debug/judgements/excel_overviews/overview_aae.xlsx
+++ b/debug/judgements/excel_overviews/overview_aae.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="335">
   <si>
     <t>vs_Llama-2-7b-chat-hf</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t>claude-haiku-4-5-20251001</t>
+  </si>
+  <si>
+    <t>claude-opus-4-5-20251101</t>
   </si>
   <si>
     <t>ASR: 0.75
@@ -109,6 +112,10 @@
 V1: 134 V2: 5 Vties: 3</t>
   </si>
   <si>
+    <t>ASR: 0.28
+V1: 127 V2: 2 Vties: 12</t>
+  </si>
+  <si>
     <t>ASR: 0.90
 V1: 80 V2: 39 Vties: 22</t>
   </si>
@@ -145,6 +152,10 @@
 V1: 96 V2: 37 Vties: 9</t>
   </si>
   <si>
+    <t>ASR: 0.41
+V1: 75 V2: 22 Vties: 42</t>
+  </si>
+  <si>
     <t>ASR: 0.79
 V1: 77 V2: 25 Vties: 33</t>
   </si>
@@ -181,6 +192,10 @@
 V1: 104 V2: 23 Vties: 15</t>
   </si>
   <si>
+    <t>ASR: 0.43
+V1: 84 V2: 12 Vties: 42</t>
+  </si>
+  <si>
     <t>ASR: 0.49
 V1: 123 V2: 7 Vties: 7</t>
   </si>
@@ -217,6 +232,10 @@
 V1: 140 V2: 0 Vties: 2</t>
   </si>
   <si>
+    <t>ASR: 0.07
+V1: 140 V2: 0 Vties: 1</t>
+  </si>
+  <si>
     <t>ASR: 0.90
 V1: 49 V2: 70 Vties: 19</t>
   </si>
@@ -253,6 +272,10 @@
 V1: 75 V2: 57 Vties: 10</t>
   </si>
   <si>
+    <t>ASR: 0.49
+V1: 67 V2: 40 Vties: 32</t>
+  </si>
+  <si>
     <t>ASR: 0.80
 V1: 101 V2: 21 Vties: 17</t>
   </si>
@@ -289,6 +312,10 @@
 V1: 128 V2: 12 Vties: 2</t>
   </si>
   <si>
+    <t>ASR: 0.41
+V1: 120 V2: 3 Vties: 15</t>
+  </si>
+  <si>
     <t>ASR: 0.89
 V1: 62 V2: 50 Vties: 22</t>
   </si>
@@ -325,6 +352,10 @@
 V1: 84 V2: 43 Vties: 15</t>
   </si>
   <si>
+    <t>ASR: 0.59
+V1: 70 V2: 19 Vties: 52</t>
+  </si>
+  <si>
     <t>ASR: 0.83
 V1: 103 V2: 11 Vties: 24</t>
   </si>
@@ -361,6 +392,10 @@
 V1: 139 V2: 2 Vties: 0</t>
   </si>
   <si>
+    <t>ASR: 0.15
+V1: 141 V2: 1 Vties: 0</t>
+  </si>
+  <si>
     <t>AASR: 0.00
 V1: 108 V2: 13 Vties: 14</t>
   </si>
@@ -393,6 +428,10 @@
 V1: 133 V2: 6 Vties: 3</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 127 V2: 2 Vties: 12</t>
+  </si>
+  <si>
     <t>AASR: 0.05
 V1: 80 V2: 39 Vties: 22</t>
   </si>
@@ -429,6 +468,10 @@
 V1: 96 V2: 37 Vties: 9</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 75 V2: 22 Vties: 42</t>
+  </si>
+  <si>
     <t>AASR: 0.08
 V1: 77 V2: 25 Vties: 33</t>
   </si>
@@ -465,6 +508,10 @@
 V1: 104 V2: 23 Vties: 15</t>
   </si>
   <si>
+    <t>AASR: 0.08
+V1: 84 V2: 12 Vties: 42</t>
+  </si>
+  <si>
     <t>AASR: 0.00
 V1: 123 V2: 7 Vties: 7</t>
   </si>
@@ -493,6 +540,10 @@
 V1: 141 V2: 0 Vties: 1</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 140 V2: 0 Vties: 1</t>
+  </si>
+  <si>
     <t>AASR: 0.03
 V1: 49 V2: 70 Vties: 19</t>
   </si>
@@ -529,6 +580,10 @@
 V1: 75 V2: 57 Vties: 10</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 67 V2: 40 Vties: 32</t>
+  </si>
+  <si>
     <t>AASR: 0.05
 V1: 101 V2: 21 Vties: 17</t>
   </si>
@@ -566,6 +621,10 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 120 V2: 3 Vties: 15</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 62 V2: 50 Vties: 22</t>
   </si>
   <si>
@@ -602,6 +661,10 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 70 V2: 19 Vties: 52</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 103 V2: 11 Vties: 24</t>
   </si>
   <si>
@@ -631,6 +694,10 @@
   <si>
     <t>AASR: 0.00
 V1: 139 V2: 2 Vties: 0</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
+V1: 141 V2: 1 Vties: 0</t>
   </si>
   <si>
     <t>FR: 0.70
@@ -669,6 +736,10 @@
 V1: 134 V2: 5 Vties: 3</t>
   </si>
   <si>
+    <t>FR: 0.33
+V1: 127 V2: 2 Vties: 12</t>
+  </si>
+  <si>
     <t>FR: 0.68
 V1: 80 V2: 39 Vties: 22</t>
   </si>
@@ -705,6 +776,10 @@
 V1: 96 V2: 37 Vties: 9</t>
   </si>
   <si>
+    <t>FR: 0.53
+V1: 75 V2: 22 Vties: 42</t>
+  </si>
+  <si>
     <t>FR: 0.71
 V1: 77 V2: 25 Vties: 33</t>
   </si>
@@ -741,6 +816,10 @@
 V1: 104 V2: 23 Vties: 15</t>
   </si>
   <si>
+    <t>FR: 0.57
+V1: 84 V2: 12 Vties: 42</t>
+  </si>
+  <si>
     <t>FR: 0.49
 V1: 123 V2: 7 Vties: 7</t>
   </si>
@@ -777,6 +856,10 @@
 V1: 140 V2: 0 Vties: 2</t>
   </si>
   <si>
+    <t>FR: 0.08
+V1: 140 V2: 0 Vties: 1</t>
+  </si>
+  <si>
     <t>FR: 0.47
 V1: 49 V2: 70 Vties: 19</t>
   </si>
@@ -813,6 +896,10 @@
 V1: 75 V2: 57 Vties: 10</t>
   </si>
   <si>
+    <t>FR: 0.47
+V1: 67 V2: 40 Vties: 32</t>
+  </si>
+  <si>
     <t>FR: 0.71
 V1: 101 V2: 21 Vties: 17</t>
   </si>
@@ -849,6 +936,10 @@
 V1: 128 V2: 12 Vties: 2</t>
   </si>
   <si>
+    <t>FR: 0.46
+V1: 120 V2: 3 Vties: 15</t>
+  </si>
+  <si>
     <t>FR: 0.57
 V1: 62 V2: 50 Vties: 22</t>
   </si>
@@ -885,6 +976,10 @@
 V1: 84 V2: 43 Vties: 15</t>
   </si>
   <si>
+    <t>FR: 0.66
+V1: 70 V2: 19 Vties: 52</t>
+  </si>
+  <si>
     <t>FR: 0.80
 V1: 103 V2: 11 Vties: 24</t>
   </si>
@@ -921,6 +1016,10 @@
 V1: 139 V2: 2 Vties: 0</t>
   </si>
   <si>
+    <t>FR: 0.15
+V1: 141 V2: 1 Vties: 0</t>
+  </si>
+  <si>
     <t>CR: 0.33
 V1: 108 V2: 13 Vties: 14</t>
   </si>
@@ -957,6 +1056,10 @@
 V1: 134 V2: 5 Vties: 3</t>
   </si>
   <si>
+    <t>CR: 0.73
+V1: 127 V2: 2 Vties: 12</t>
+  </si>
+  <si>
     <t>CR: 0.38
 V1: 80 V2: 39 Vties: 22</t>
   </si>
@@ -993,6 +1096,10 @@
 V1: 96 V2: 37 Vties: 9</t>
   </si>
   <si>
+    <t>CR: 0.68
+V1: 75 V2: 22 Vties: 42</t>
+  </si>
+  <si>
     <t>CR: 0.38
 V1: 77 V2: 25 Vties: 33</t>
   </si>
@@ -1029,6 +1136,10 @@
 V1: 104 V2: 23 Vties: 15</t>
   </si>
   <si>
+    <t>CR: 0.61
+V1: 84 V2: 12 Vties: 42</t>
+  </si>
+  <si>
     <t>CR: 0.54
 V1: 123 V2: 7 Vties: 7</t>
   </si>
@@ -1065,6 +1176,10 @@
 V1: 140 V2: 0 Vties: 2</t>
   </si>
   <si>
+    <t>CR: 0.93
+V1: 140 V2: 0 Vties: 1</t>
+  </si>
+  <si>
     <t>CR: 0.61
 V1: 49 V2: 70 Vties: 19</t>
   </si>
@@ -1101,6 +1216,10 @@
 V1: 75 V2: 57 Vties: 10</t>
   </si>
   <si>
+    <t>CR: 0.69
+V1: 67 V2: 40 Vties: 32</t>
+  </si>
+  <si>
     <t>CR: 0.33
 V1: 101 V2: 21 Vties: 17</t>
   </si>
@@ -1137,6 +1256,10 @@
 V1: 128 V2: 12 Vties: 2</t>
   </si>
   <si>
+    <t>CR: 0.60
+V1: 120 V2: 3 Vties: 15</t>
+  </si>
+  <si>
     <t>CR: 0.51
 V1: 62 V2: 50 Vties: 22</t>
   </si>
@@ -1173,6 +1296,10 @@
 V1: 84 V2: 43 Vties: 15</t>
   </si>
   <si>
+    <t>CR: 0.54
+V1: 70 V2: 19 Vties: 52</t>
+  </si>
+  <si>
     <t>CR: 0.25
 V1: 103 V2: 11 Vties: 24</t>
   </si>
@@ -1207,6 +1334,10 @@
   <si>
     <t>CR: 0.53
 V1: 139 V2: 2 Vties: 0</t>
+  </si>
+  <si>
+    <t>CR: 0.85
+V1: 141 V2: 1 Vties: 0</t>
   </si>
 </sst>
 </file>
@@ -1567,7 +1698,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
@@ -1607,28 +1738,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1636,28 +1767,28 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1665,28 +1796,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1694,28 +1825,28 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1723,28 +1854,28 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1752,28 +1883,28 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1781,28 +1912,28 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1810,28 +1941,28 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1839,28 +1970,57 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>89</v>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1870,7 +2030,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
@@ -1910,28 +2070,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1939,28 +2099,28 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1968,28 +2128,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1997,28 +2157,28 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2026,28 +2186,28 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2055,28 +2215,28 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2084,28 +2244,28 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2113,28 +2273,28 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2142,28 +2302,57 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>149</v>
+        <v>164</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>157</v>
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2173,7 +2362,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
@@ -2213,28 +2402,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2242,28 +2431,28 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>213</v>
+        <v>236</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2271,28 +2460,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>205</v>
+        <v>227</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>214</v>
+        <v>237</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>223</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2300,28 +2489,28 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>215</v>
+        <v>238</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>224</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2329,28 +2518,28 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>207</v>
+        <v>229</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>216</v>
+        <v>239</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>225</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2358,28 +2547,28 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>208</v>
+        <v>230</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>217</v>
+        <v>240</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>226</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2387,28 +2576,28 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>209</v>
+        <v>231</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>218</v>
+        <v>241</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>227</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2416,28 +2605,28 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>192</v>
+        <v>212</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>210</v>
+        <v>232</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>219</v>
+        <v>242</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>228</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2445,28 +2634,57 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>229</v>
+      <c r="C11" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -2476,7 +2694,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
@@ -2516,28 +2734,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>230</v>
+        <v>255</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>239</v>
+        <v>265</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>248</v>
+        <v>275</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>257</v>
+        <v>285</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>266</v>
+        <v>295</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>284</v>
+        <v>315</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>293</v>
+        <v>325</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2545,28 +2763,28 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>240</v>
+        <v>266</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>249</v>
+        <v>276</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>258</v>
+        <v>286</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>267</v>
+        <v>296</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>276</v>
+        <v>306</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>285</v>
+        <v>316</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>294</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2574,28 +2792,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>232</v>
+        <v>257</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>241</v>
+        <v>267</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>250</v>
+        <v>277</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>259</v>
+        <v>287</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>268</v>
+        <v>297</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>277</v>
+        <v>307</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>286</v>
+        <v>317</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>295</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2603,28 +2821,28 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>233</v>
+        <v>258</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>242</v>
+        <v>268</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>251</v>
+        <v>278</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>260</v>
+        <v>288</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>269</v>
+        <v>298</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>278</v>
+        <v>308</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>287</v>
+        <v>318</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>296</v>
+        <v>328</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2632,28 +2850,28 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>234</v>
+        <v>259</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>243</v>
+        <v>269</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>252</v>
+        <v>279</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>261</v>
+        <v>289</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>270</v>
+        <v>299</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>279</v>
+        <v>309</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>288</v>
+        <v>319</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>297</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2661,28 +2879,28 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>235</v>
+        <v>260</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>244</v>
+        <v>270</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>253</v>
+        <v>280</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>262</v>
+        <v>290</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>271</v>
+        <v>300</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>280</v>
+        <v>310</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>289</v>
+        <v>320</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>298</v>
+        <v>330</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2690,28 +2908,28 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>236</v>
+        <v>261</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>245</v>
+        <v>271</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>254</v>
+        <v>281</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>263</v>
+        <v>291</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>281</v>
+        <v>311</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>290</v>
+        <v>321</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>299</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2719,28 +2937,28 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>237</v>
+        <v>262</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>246</v>
+        <v>272</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>255</v>
+        <v>282</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>264</v>
+        <v>292</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>282</v>
+        <v>312</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>291</v>
+        <v>322</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>300</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2748,28 +2966,57 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>238</v>
+        <v>263</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>247</v>
+        <v>273</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>256</v>
+        <v>283</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>265</v>
+        <v>293</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>301</v>
+      <c r="D11" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Gemini 2.5 Pro Judgements
</commit_message>
<xml_diff>
--- a/debug/judgements/excel_overviews/overview_aae.xlsx
+++ b/debug/judgements/excel_overviews/overview_aae.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="368">
   <si>
     <t>vs_Llama-2-7b-chat-hf</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t>claude-opus-4-5-20251101</t>
+  </si>
+  <si>
+    <t>gemini-2.5-pro</t>
   </si>
   <si>
     <t>ASR: 0.75
@@ -116,6 +119,10 @@
 V1: 127 V2: 2 Vties: 12</t>
   </si>
   <si>
+    <t>ASR: 0.26
+V1: 133 V2: 4 Vties: 5</t>
+  </si>
+  <si>
     <t>ASR: 0.90
 V1: 80 V2: 39 Vties: 22</t>
   </si>
@@ -156,6 +163,10 @@
 V1: 75 V2: 22 Vties: 42</t>
   </si>
   <si>
+    <t>ASR: 0.50
+V1: 90 V2: 26 Vties: 26</t>
+  </si>
+  <si>
     <t>ASR: 0.79
 V1: 77 V2: 25 Vties: 33</t>
   </si>
@@ -196,6 +207,10 @@
 V1: 84 V2: 12 Vties: 42</t>
   </si>
   <si>
+    <t>ASR: 0.58
+V1: 102 V2: 14 Vties: 26</t>
+  </si>
+  <si>
     <t>ASR: 0.49
 V1: 123 V2: 7 Vties: 7</t>
   </si>
@@ -236,6 +251,10 @@
 V1: 140 V2: 0 Vties: 1</t>
   </si>
   <si>
+    <t>ASR: 0.09
+V1: 142 V2: 0 Vties: 0</t>
+  </si>
+  <si>
     <t>ASR: 0.90
 V1: 49 V2: 70 Vties: 19</t>
   </si>
@@ -276,6 +295,10 @@
 V1: 67 V2: 40 Vties: 32</t>
   </si>
   <si>
+    <t>ASR: 0.67
+V1: 66 V2: 47 Vties: 29</t>
+  </si>
+  <si>
     <t>ASR: 0.80
 V1: 101 V2: 21 Vties: 17</t>
   </si>
@@ -316,6 +339,10 @@
 V1: 120 V2: 3 Vties: 15</t>
   </si>
   <si>
+    <t>ASR: 0.38
+V1: 125 V2: 6 Vties: 11</t>
+  </si>
+  <si>
     <t>ASR: 0.89
 V1: 62 V2: 50 Vties: 22</t>
   </si>
@@ -356,6 +383,10 @@
 V1: 70 V2: 19 Vties: 52</t>
   </si>
   <si>
+    <t>ASR: 0.66
+V1: 79 V2: 28 Vties: 35</t>
+  </si>
+  <si>
     <t>ASR: 0.83
 V1: 103 V2: 11 Vties: 24</t>
   </si>
@@ -396,6 +427,10 @@
 V1: 141 V2: 1 Vties: 0</t>
   </si>
   <si>
+    <t>ASR: 0.19
+V1: 139 V2: 0 Vties: 3</t>
+  </si>
+  <si>
     <t>AASR: 0.00
 V1: 108 V2: 13 Vties: 14</t>
   </si>
@@ -432,6 +467,10 @@
 V1: 127 V2: 2 Vties: 12</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 133 V2: 4 Vties: 5</t>
+  </si>
+  <si>
     <t>AASR: 0.05
 V1: 80 V2: 39 Vties: 22</t>
   </si>
@@ -472,6 +511,10 @@
 V1: 75 V2: 22 Vties: 42</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 90 V2: 26 Vties: 26</t>
+  </si>
+  <si>
     <t>AASR: 0.08
 V1: 77 V2: 25 Vties: 33</t>
   </si>
@@ -513,6 +556,10 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 102 V2: 14 Vties: 26</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 123 V2: 7 Vties: 7</t>
   </si>
   <si>
@@ -544,6 +591,10 @@
 V1: 140 V2: 0 Vties: 1</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 142 V2: 0 Vties: 0</t>
+  </si>
+  <si>
     <t>AASR: 0.03
 V1: 49 V2: 70 Vties: 19</t>
   </si>
@@ -584,6 +635,10 @@
 V1: 67 V2: 40 Vties: 32</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 66 V2: 47 Vties: 29</t>
+  </si>
+  <si>
     <t>AASR: 0.05
 V1: 101 V2: 21 Vties: 17</t>
   </si>
@@ -625,6 +680,10 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 125 V2: 6 Vties: 11</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 62 V2: 50 Vties: 22</t>
   </si>
   <si>
@@ -665,6 +724,10 @@
   </si>
   <si>
     <t>AASR: 0.00
+V1: 79 V2: 28 Vties: 35</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
 V1: 103 V2: 11 Vties: 24</t>
   </si>
   <si>
@@ -698,6 +761,10 @@
   <si>
     <t>AASR: 0.00
 V1: 141 V2: 1 Vties: 0</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
+V1: 139 V2: 0 Vties: 3</t>
   </si>
   <si>
     <t>FR: 0.70
@@ -740,6 +807,10 @@
 V1: 127 V2: 2 Vties: 12</t>
   </si>
   <si>
+    <t>FR: 0.27
+V1: 133 V2: 4 Vties: 5</t>
+  </si>
+  <si>
     <t>FR: 0.68
 V1: 80 V2: 39 Vties: 22</t>
   </si>
@@ -780,6 +851,10 @@
 V1: 75 V2: 22 Vties: 42</t>
   </si>
   <si>
+    <t>FR: 0.50
+V1: 90 V2: 26 Vties: 26</t>
+  </si>
+  <si>
     <t>FR: 0.71
 V1: 77 V2: 25 Vties: 33</t>
   </si>
@@ -820,6 +895,10 @@
 V1: 84 V2: 12 Vties: 42</t>
   </si>
   <si>
+    <t>FR: 0.60
+V1: 102 V2: 14 Vties: 26</t>
+  </si>
+  <si>
     <t>FR: 0.49
 V1: 123 V2: 7 Vties: 7</t>
   </si>
@@ -860,6 +939,10 @@
 V1: 140 V2: 0 Vties: 1</t>
   </si>
   <si>
+    <t>FR: 0.09
+V1: 142 V2: 0 Vties: 0</t>
+  </si>
+  <si>
     <t>FR: 0.47
 V1: 49 V2: 70 Vties: 19</t>
   </si>
@@ -900,6 +983,10 @@
 V1: 67 V2: 40 Vties: 32</t>
   </si>
   <si>
+    <t>FR: 0.51
+V1: 66 V2: 47 Vties: 29</t>
+  </si>
+  <si>
     <t>FR: 0.71
 V1: 101 V2: 21 Vties: 17</t>
   </si>
@@ -940,6 +1027,10 @@
 V1: 120 V2: 3 Vties: 15</t>
   </si>
   <si>
+    <t>FR: 0.42
+V1: 125 V2: 6 Vties: 11</t>
+  </si>
+  <si>
     <t>FR: 0.57
 V1: 62 V2: 50 Vties: 22</t>
   </si>
@@ -980,6 +1071,10 @@
 V1: 70 V2: 19 Vties: 52</t>
   </si>
   <si>
+    <t>FR: 0.61
+V1: 79 V2: 28 Vties: 35</t>
+  </si>
+  <si>
     <t>FR: 0.80
 V1: 103 V2: 11 Vties: 24</t>
   </si>
@@ -1020,6 +1115,10 @@
 V1: 141 V2: 1 Vties: 0</t>
   </si>
   <si>
+    <t>FR: 0.21
+V1: 139 V2: 0 Vties: 3</t>
+  </si>
+  <si>
     <t>CR: 0.33
 V1: 108 V2: 13 Vties: 14</t>
   </si>
@@ -1060,6 +1159,10 @@
 V1: 127 V2: 2 Vties: 12</t>
   </si>
   <si>
+    <t>CR: 0.75
+V1: 133 V2: 4 Vties: 5</t>
+  </si>
+  <si>
     <t>CR: 0.38
 V1: 80 V2: 39 Vties: 22</t>
   </si>
@@ -1100,6 +1203,10 @@
 V1: 75 V2: 22 Vties: 42</t>
   </si>
   <si>
+    <t>CR: 0.61
+V1: 90 V2: 26 Vties: 26</t>
+  </si>
+  <si>
     <t>CR: 0.38
 V1: 77 V2: 25 Vties: 33</t>
   </si>
@@ -1140,6 +1247,10 @@
 V1: 84 V2: 12 Vties: 42</t>
   </si>
   <si>
+    <t>CR: 0.49
+V1: 102 V2: 14 Vties: 26</t>
+  </si>
+  <si>
     <t>CR: 0.54
 V1: 123 V2: 7 Vties: 7</t>
   </si>
@@ -1180,6 +1291,10 @@
 V1: 140 V2: 0 Vties: 1</t>
   </si>
   <si>
+    <t>CR: 0.91
+V1: 142 V2: 0 Vties: 0</t>
+  </si>
+  <si>
     <t>CR: 0.61
 V1: 49 V2: 70 Vties: 19</t>
   </si>
@@ -1220,6 +1335,10 @@
 V1: 67 V2: 40 Vties: 32</t>
   </si>
   <si>
+    <t>CR: 0.61
+V1: 66 V2: 47 Vties: 29</t>
+  </si>
+  <si>
     <t>CR: 0.33
 V1: 101 V2: 21 Vties: 17</t>
   </si>
@@ -1260,6 +1379,10 @@
 V1: 120 V2: 3 Vties: 15</t>
   </si>
   <si>
+    <t>CR: 0.63
+V1: 125 V2: 6 Vties: 11</t>
+  </si>
+  <si>
     <t>CR: 0.51
 V1: 62 V2: 50 Vties: 22</t>
   </si>
@@ -1300,6 +1423,10 @@
 V1: 70 V2: 19 Vties: 52</t>
   </si>
   <si>
+    <t>CR: 0.51
+V1: 79 V2: 28 Vties: 35</t>
+  </si>
+  <si>
     <t>CR: 0.25
 V1: 103 V2: 11 Vties: 24</t>
   </si>
@@ -1338,6 +1465,10 @@
   <si>
     <t>CR: 0.85
 V1: 141 V2: 1 Vties: 0</t>
+  </si>
+  <si>
+    <t>CR: 0.81
+V1: 139 V2: 0 Vties: 3</t>
   </si>
 </sst>
 </file>
@@ -1698,7 +1829,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
@@ -1738,28 +1869,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1767,28 +1898,28 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1796,28 +1927,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1825,28 +1956,28 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1854,28 +1985,28 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1883,28 +2014,28 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1912,28 +2043,28 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1941,28 +2072,28 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1970,28 +2101,28 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1999,28 +2130,57 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2030,7 +2190,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
@@ -2070,28 +2230,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2099,28 +2259,28 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2128,28 +2288,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2157,28 +2317,28 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2186,28 +2346,28 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2215,28 +2375,28 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2244,28 +2404,28 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2273,28 +2433,28 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2302,28 +2462,28 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -2331,28 +2491,57 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>174</v>
+      <c r="C12" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -2362,7 +2551,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
@@ -2402,28 +2591,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>205</v>
+        <v>225</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>225</v>
+        <v>247</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>235</v>
+        <v>258</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>245</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2431,28 +2620,28 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>206</v>
+        <v>226</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>216</v>
+        <v>237</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>236</v>
+        <v>259</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>246</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2460,28 +2649,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>207</v>
+        <v>227</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>227</v>
+        <v>249</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>237</v>
+        <v>260</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>247</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2489,28 +2678,28 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>178</v>
+        <v>195</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>188</v>
+        <v>206</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>228</v>
+        <v>250</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>238</v>
+        <v>261</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>248</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2518,28 +2707,28 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>209</v>
+        <v>229</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>229</v>
+        <v>251</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>239</v>
+        <v>262</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>249</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2547,28 +2736,28 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>190</v>
+        <v>208</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>230</v>
+        <v>252</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>240</v>
+        <v>263</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>250</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2576,28 +2765,28 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>181</v>
+        <v>198</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>191</v>
+        <v>209</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>211</v>
+        <v>231</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>221</v>
+        <v>242</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>241</v>
+        <v>264</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>251</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2605,28 +2794,28 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>182</v>
+        <v>199</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>192</v>
+        <v>210</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>212</v>
+        <v>232</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>222</v>
+        <v>243</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>232</v>
+        <v>254</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>242</v>
+        <v>265</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2634,28 +2823,28 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>183</v>
+        <v>200</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>243</v>
+        <v>266</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>253</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -2663,28 +2852,57 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>184</v>
+        <v>201</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
       <c r="F11" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>254</v>
+      <c r="E12" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -2694,7 +2912,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
@@ -2734,28 +2952,28 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>255</v>
+        <v>280</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>265</v>
+        <v>291</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>275</v>
+        <v>302</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>285</v>
+        <v>313</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>295</v>
+        <v>324</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>305</v>
+        <v>335</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>315</v>
+        <v>346</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>325</v>
+        <v>357</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2763,28 +2981,28 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>256</v>
+        <v>281</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>266</v>
+        <v>292</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>276</v>
+        <v>303</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>286</v>
+        <v>314</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>296</v>
+        <v>325</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>306</v>
+        <v>336</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>316</v>
+        <v>347</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>326</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2792,28 +3010,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>267</v>
+        <v>293</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>277</v>
+        <v>304</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>287</v>
+        <v>315</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>297</v>
+        <v>326</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>307</v>
+        <v>337</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>317</v>
+        <v>348</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>327</v>
+        <v>359</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2821,28 +3039,28 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>258</v>
+        <v>283</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>268</v>
+        <v>294</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>278</v>
+        <v>305</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>288</v>
+        <v>316</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>298</v>
+        <v>327</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>308</v>
+        <v>338</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>318</v>
+        <v>349</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>328</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2850,28 +3068,28 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>269</v>
+        <v>295</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>279</v>
+        <v>306</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>289</v>
+        <v>317</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>299</v>
+        <v>328</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>309</v>
+        <v>339</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>319</v>
+        <v>350</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>329</v>
+        <v>361</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2879,28 +3097,28 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>260</v>
+        <v>285</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>270</v>
+        <v>296</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>280</v>
+        <v>307</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>290</v>
+        <v>318</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>300</v>
+        <v>329</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>310</v>
+        <v>340</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>320</v>
+        <v>351</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>330</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2908,28 +3126,28 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>261</v>
+        <v>286</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>271</v>
+        <v>297</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>281</v>
+        <v>308</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>291</v>
+        <v>319</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>301</v>
+        <v>330</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>311</v>
+        <v>341</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>321</v>
+        <v>352</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>331</v>
+        <v>363</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2937,28 +3155,28 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>262</v>
+        <v>287</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>272</v>
+        <v>298</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>282</v>
+        <v>309</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>292</v>
+        <v>320</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>302</v>
+        <v>331</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>312</v>
+        <v>342</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>322</v>
+        <v>353</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>332</v>
+        <v>364</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2966,28 +3184,28 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>263</v>
+        <v>288</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>273</v>
+        <v>299</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>283</v>
+        <v>310</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>293</v>
+        <v>321</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>303</v>
+        <v>332</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>313</v>
+        <v>343</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>323</v>
+        <v>354</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>333</v>
+        <v>365</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -2995,28 +3213,57 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>264</v>
+        <v>289</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>284</v>
+        <v>311</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>294</v>
+        <v>322</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>304</v>
+        <v>333</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>314</v>
+        <v>344</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>324</v>
+        <v>355</v>
       </c>
       <c r="I11" s="1" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>334</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>